<commit_message>
workbook: no number-stored-as-text warnings on label columns
</commit_message>
<xml_diff>
--- a/output/inventory_health_check.xlsx
+++ b/output/inventory_health_check.xlsx
@@ -38620,6 +38620,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="B2:B110" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -44932,6 +44935,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A2:A140" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 

</xml_diff>